<commit_message>
add dataset and update scripts
add dataset and update scripts
</commit_message>
<xml_diff>
--- a/data/result_for_figure.xlsx
+++ b/data/result_for_figure.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10905"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhiyuanzhang/Downloads/PPIpredictHumanVirus/paperdataset/binaryPPI_paper/result/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhiyuanzhang/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885FADE5-854E-A945-9B41-FF6B4E9389A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E1F3EED-8C6B-1F42-A832-BDA513579B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34600" yWindow="1460" windowWidth="25820" windowHeight="16280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2160" yWindow="500" windowWidth="25820" windowHeight="16280" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="paperdataset_test_auroc" sheetId="2" r:id="rId1"/>
     <sheet name="mydataset_test_auroc" sheetId="3" r:id="rId2"/>
+    <sheet name="mydataset_test_acc_auroc_auprc" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="14">
   <si>
     <t>Paper</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -54,6 +55,27 @@
   <si>
     <t>PPI-Top450-RF</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Genome-3mer-RF</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Accuracy</t>
+  </si>
+  <si>
+    <t>AUROC</t>
+  </si>
+  <si>
+    <t>AUPRC</t>
+  </si>
+  <si>
+    <t>Proteome-esm2-RF</t>
+  </si>
+  <si>
+    <t>PPI-Top450-RF</t>
   </si>
 </sst>
 </file>
@@ -2941,4 +2963,4234 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AC2FF46-6733-9D45-B769-B8ACAE7551C6}">
+  <dimension ref="A1:D301"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.1640625" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2">
+        <v>0.73056994818652798</v>
+      </c>
+      <c r="C2">
+        <v>0.69948186528497402</v>
+      </c>
+      <c r="D2">
+        <v>0.76165803108808205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="C3">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="D3">
+        <v>0.77720207253885998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="C4">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D4">
+        <v>0.76683937823834103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="C5">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D5">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>0.71502590673575095</v>
+      </c>
+      <c r="C6">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D6">
+        <v>0.79792746113989599</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C7">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="D7">
+        <v>0.80310880829015496</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>0.74093264248704604</v>
+      </c>
+      <c r="C8">
+        <v>0.73056994818652798</v>
+      </c>
+      <c r="D8">
+        <v>0.818652849740932</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C9">
+        <v>0.74093264248704604</v>
+      </c>
+      <c r="D9">
+        <v>0.72538860103626901</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C10">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="D10">
+        <v>0.72538860103626901</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>0.80310880829015496</v>
+      </c>
+      <c r="C11">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="D11">
+        <v>0.79792746113989599</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="C12">
+        <v>0.72020725388601003</v>
+      </c>
+      <c r="D12">
+        <v>0.78238341968911895</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="C13">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D13">
+        <v>0.78238341968911895</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>0.75129533678756399</v>
+      </c>
+      <c r="C14">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D14">
+        <v>0.75129533678756399</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="C15">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="D15">
+        <v>0.76165803108808205</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C16">
+        <v>0.704663212435233</v>
+      </c>
+      <c r="D16">
+        <v>0.79274611398963701</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17">
+        <v>0.74093264248704604</v>
+      </c>
+      <c r="C17">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="D17">
+        <v>0.772020725388601</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18">
+        <v>0.72538860103626901</v>
+      </c>
+      <c r="C18">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="D18">
+        <v>0.79792746113989599</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="C19">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="D19">
+        <v>0.78238341968911895</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="C20">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="D20">
+        <v>0.75647668393782297</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21">
+        <v>0.75129533678756399</v>
+      </c>
+      <c r="C21">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D21">
+        <v>0.79274611398963701</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="C22">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="D22">
+        <v>0.75647668393782297</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="C23">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D23">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C24">
+        <v>0.80310880829015496</v>
+      </c>
+      <c r="D24">
+        <v>0.76165803108808205</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C25">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="D25">
+        <v>0.76683937823834103</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26">
+        <v>0.75129533678756399</v>
+      </c>
+      <c r="C26">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="D26">
+        <v>0.77720207253885998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="C27">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="D27">
+        <v>0.82901554404144995</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="C28">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D28">
+        <v>0.76683937823834103</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="C29">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="D29">
+        <v>0.79792746113989599</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30">
+        <v>0.75129533678756399</v>
+      </c>
+      <c r="C30">
+        <v>0.72538860103626901</v>
+      </c>
+      <c r="D30">
+        <v>0.75647668393782297</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="C31">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="D31">
+        <v>0.77720207253885998</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32">
+        <v>0.72538860103626901</v>
+      </c>
+      <c r="C32">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="D32">
+        <v>0.76165803108808205</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" t="s">
+        <v>9</v>
+      </c>
+      <c r="B33">
+        <v>0.80310880829015496</v>
+      </c>
+      <c r="C33">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="D33">
+        <v>0.74611398963730502</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34">
+        <v>0.70984455958549197</v>
+      </c>
+      <c r="C34">
+        <v>0.71502590673575095</v>
+      </c>
+      <c r="D34">
+        <v>0.83937823834196801</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="C35">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D35">
+        <v>0.77720207253885998</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C36">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="D36">
+        <v>0.80829015544041405</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37">
+        <v>0.75129533678756399</v>
+      </c>
+      <c r="C37">
+        <v>0.78238341968911895</v>
+      </c>
+      <c r="D37">
+        <v>0.82383419689119097</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="C38">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="D38">
+        <v>0.79274611398963701</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39">
+        <v>0.73056994818652798</v>
+      </c>
+      <c r="C39">
+        <v>0.79792746113989599</v>
+      </c>
+      <c r="D39">
+        <v>0.772020725388601</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>9</v>
+      </c>
+      <c r="B40">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="C40">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D40">
+        <v>0.74093264248704604</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B41">
+        <v>0.72538860103626901</v>
+      </c>
+      <c r="C41">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="D41">
+        <v>0.80310880829015496</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42">
+        <v>0.71502590673575095</v>
+      </c>
+      <c r="C42">
+        <v>0.69430051813471505</v>
+      </c>
+      <c r="D42">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>9</v>
+      </c>
+      <c r="B43">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C43">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="D43">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" t="s">
+        <v>9</v>
+      </c>
+      <c r="B44">
+        <v>0.80310880829015496</v>
+      </c>
+      <c r="C44">
+        <v>0.81347150259067302</v>
+      </c>
+      <c r="D44">
+        <v>0.80310880829015496</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" t="s">
+        <v>9</v>
+      </c>
+      <c r="B45">
+        <v>0.74093264248704604</v>
+      </c>
+      <c r="C45">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D45">
+        <v>0.78238341968911895</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" t="s">
+        <v>9</v>
+      </c>
+      <c r="B46">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="C46">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="D46">
+        <v>0.81347150259067302</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47">
+        <v>0.80310880829015496</v>
+      </c>
+      <c r="C47">
+        <v>0.82383419689119097</v>
+      </c>
+      <c r="D47">
+        <v>0.73575129533678696</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" t="s">
+        <v>9</v>
+      </c>
+      <c r="B48">
+        <v>0.80310880829015496</v>
+      </c>
+      <c r="C48">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="D48">
+        <v>0.76683937823834103</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" t="s">
+        <v>9</v>
+      </c>
+      <c r="B49">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="C49">
+        <v>0.75129533678756399</v>
+      </c>
+      <c r="D49">
+        <v>0.76683937823834103</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" t="s">
+        <v>9</v>
+      </c>
+      <c r="B50">
+        <v>0.72020725388601003</v>
+      </c>
+      <c r="C50">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="D50">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" t="s">
+        <v>9</v>
+      </c>
+      <c r="B51">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="C51">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="D51">
+        <v>0.75647668393782297</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" t="s">
+        <v>9</v>
+      </c>
+      <c r="B52">
+        <v>0.79792746113989599</v>
+      </c>
+      <c r="C52">
+        <v>0.80310880829015496</v>
+      </c>
+      <c r="D52">
+        <v>0.75647668393782297</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" t="s">
+        <v>9</v>
+      </c>
+      <c r="B53">
+        <v>0.78238341968911895</v>
+      </c>
+      <c r="C53">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="D53">
+        <v>0.79792746113989599</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" t="s">
+        <v>9</v>
+      </c>
+      <c r="B54">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="C54">
+        <v>0.71502590673575095</v>
+      </c>
+      <c r="D54">
+        <v>0.75647668393782297</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" t="s">
+        <v>9</v>
+      </c>
+      <c r="B55">
+        <v>0.69948186528497402</v>
+      </c>
+      <c r="C55">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="D55">
+        <v>0.80829015544041405</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" t="s">
+        <v>9</v>
+      </c>
+      <c r="B56">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="C56">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="D56">
+        <v>0.80829015544041405</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" t="s">
+        <v>9</v>
+      </c>
+      <c r="B57">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="C57">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="D57">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" t="s">
+        <v>9</v>
+      </c>
+      <c r="B58">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="C58">
+        <v>0.74093264248704604</v>
+      </c>
+      <c r="D58">
+        <v>0.83419689119170903</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" t="s">
+        <v>9</v>
+      </c>
+      <c r="B59">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="C59">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="D59">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" t="s">
+        <v>9</v>
+      </c>
+      <c r="B60">
+        <v>0.69948186528497402</v>
+      </c>
+      <c r="C60">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="D60">
+        <v>0.818652849740932</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" t="s">
+        <v>9</v>
+      </c>
+      <c r="B61">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="C61">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="D61">
+        <v>0.73575129533678696</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" t="s">
+        <v>9</v>
+      </c>
+      <c r="B62">
+        <v>0.74093264248704604</v>
+      </c>
+      <c r="C62">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="D62">
+        <v>0.80829015544041405</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" t="s">
+        <v>9</v>
+      </c>
+      <c r="B63">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="C63">
+        <v>0.78238341968911895</v>
+      </c>
+      <c r="D63">
+        <v>0.77720207253885998</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" t="s">
+        <v>9</v>
+      </c>
+      <c r="B64">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="C64">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D64">
+        <v>0.76165803108808205</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" t="s">
+        <v>9</v>
+      </c>
+      <c r="B65">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C65">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="D65">
+        <v>0.77720207253885998</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" t="s">
+        <v>9</v>
+      </c>
+      <c r="B66">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="C66">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D66">
+        <v>0.84974093264248696</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" t="s">
+        <v>9</v>
+      </c>
+      <c r="B67">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="C67">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="D67">
+        <v>0.75647668393782297</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" t="s">
+        <v>9</v>
+      </c>
+      <c r="B68">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="C68">
+        <v>0.74093264248704604</v>
+      </c>
+      <c r="D68">
+        <v>0.772020725388601</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" t="s">
+        <v>9</v>
+      </c>
+      <c r="B69">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="C69">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D69">
+        <v>0.82901554404144995</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" t="s">
+        <v>9</v>
+      </c>
+      <c r="B70">
+        <v>0.71502590673575095</v>
+      </c>
+      <c r="C70">
+        <v>0.72020725388601003</v>
+      </c>
+      <c r="D70">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" t="s">
+        <v>9</v>
+      </c>
+      <c r="B71">
+        <v>0.82901554404144995</v>
+      </c>
+      <c r="C71">
+        <v>0.82383419689119097</v>
+      </c>
+      <c r="D71">
+        <v>0.82383419689119097</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" t="s">
+        <v>9</v>
+      </c>
+      <c r="B72">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="C72">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="D72">
+        <v>0.80829015544041405</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" t="s">
+        <v>9</v>
+      </c>
+      <c r="B73">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C73">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D73">
+        <v>0.80310880829015496</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" t="s">
+        <v>9</v>
+      </c>
+      <c r="B74">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="C74">
+        <v>0.69948186528497402</v>
+      </c>
+      <c r="D74">
+        <v>0.82383419689119097</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="A75" t="s">
+        <v>9</v>
+      </c>
+      <c r="B75">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C75">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D75">
+        <v>0.76683937823834103</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="A76" t="s">
+        <v>9</v>
+      </c>
+      <c r="B76">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="C76">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D76">
+        <v>0.77720207253885998</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="A77" t="s">
+        <v>9</v>
+      </c>
+      <c r="B77">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="C77">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="D77">
+        <v>0.82383419689119097</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78" t="s">
+        <v>9</v>
+      </c>
+      <c r="B78">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C78">
+        <v>0.80310880829015496</v>
+      </c>
+      <c r="D78">
+        <v>0.74611398963730502</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79" t="s">
+        <v>9</v>
+      </c>
+      <c r="B79">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C79">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D79">
+        <v>0.73575129533678696</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" t="s">
+        <v>9</v>
+      </c>
+      <c r="B80">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="C80">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="D80">
+        <v>0.82901554404144995</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
+      <c r="A81" t="s">
+        <v>9</v>
+      </c>
+      <c r="B81">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="C81">
+        <v>0.78238341968911895</v>
+      </c>
+      <c r="D81">
+        <v>0.79792746113989599</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
+      <c r="A82" t="s">
+        <v>9</v>
+      </c>
+      <c r="B82">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="C82">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="D82">
+        <v>0.772020725388601</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
+      <c r="A83" t="s">
+        <v>9</v>
+      </c>
+      <c r="B83">
+        <v>0.75129533678756399</v>
+      </c>
+      <c r="C83">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D83">
+        <v>0.76683937823834103</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
+      <c r="A84" t="s">
+        <v>9</v>
+      </c>
+      <c r="B84">
+        <v>0.80829015544041405</v>
+      </c>
+      <c r="C84">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="D84">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
+      <c r="A85" t="s">
+        <v>9</v>
+      </c>
+      <c r="B85">
+        <v>0.72020725388601003</v>
+      </c>
+      <c r="C85">
+        <v>0.73575129533678696</v>
+      </c>
+      <c r="D85">
+        <v>0.78238341968911895</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86" t="s">
+        <v>9</v>
+      </c>
+      <c r="B86">
+        <v>0.78238341968911895</v>
+      </c>
+      <c r="C86">
+        <v>0.79792746113989599</v>
+      </c>
+      <c r="D86">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
+      <c r="A87" t="s">
+        <v>9</v>
+      </c>
+      <c r="B87">
+        <v>0.818652849740932</v>
+      </c>
+      <c r="C87">
+        <v>0.78238341968911895</v>
+      </c>
+      <c r="D87">
+        <v>0.78238341968911895</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
+      <c r="A88" t="s">
+        <v>9</v>
+      </c>
+      <c r="B88">
+        <v>0.75129533678756399</v>
+      </c>
+      <c r="C88">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="D88">
+        <v>0.772020725388601</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
+      <c r="A89" t="s">
+        <v>9</v>
+      </c>
+      <c r="B89">
+        <v>0.71502590673575095</v>
+      </c>
+      <c r="C89">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="D89">
+        <v>0.75647668393782297</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90" t="s">
+        <v>9</v>
+      </c>
+      <c r="B90">
+        <v>0.76165803108808205</v>
+      </c>
+      <c r="C90">
+        <v>0.75647668393782297</v>
+      </c>
+      <c r="D90">
+        <v>0.78238341968911895</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
+      <c r="A91" t="s">
+        <v>9</v>
+      </c>
+      <c r="B91">
+        <v>0.80310880829015496</v>
+      </c>
+      <c r="C91">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="D91">
+        <v>0.79792746113989599</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
+      <c r="A92" t="s">
+        <v>9</v>
+      </c>
+      <c r="B92">
+        <v>0.772020725388601</v>
+      </c>
+      <c r="C92">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="D92">
+        <v>0.78238341968911895</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93" t="s">
+        <v>9</v>
+      </c>
+      <c r="B93">
+        <v>0.73056994818652798</v>
+      </c>
+      <c r="C93">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="D93">
+        <v>0.77720207253885998</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
+      <c r="A94" t="s">
+        <v>9</v>
+      </c>
+      <c r="B94">
+        <v>0.73056994818652798</v>
+      </c>
+      <c r="C94">
+        <v>0.74611398963730502</v>
+      </c>
+      <c r="D94">
+        <v>0.79792746113989599</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
+      <c r="A95" t="s">
+        <v>9</v>
+      </c>
+      <c r="B95">
+        <v>0.80829015544041405</v>
+      </c>
+      <c r="C95">
+        <v>0.818652849740932</v>
+      </c>
+      <c r="D95">
+        <v>0.75647668393782297</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
+      <c r="A96" t="s">
+        <v>9</v>
+      </c>
+      <c r="B96">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="C96">
+        <v>0.79274611398963701</v>
+      </c>
+      <c r="D96">
+        <v>0.78756476683937804</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
+      <c r="A97" t="s">
+        <v>9</v>
+      </c>
+      <c r="B97">
+        <v>0.73056994818652798</v>
+      </c>
+      <c r="C97">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="D97">
+        <v>0.79792746113989599</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
+      <c r="A98" t="s">
+        <v>9</v>
+      </c>
+      <c r="B98">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="C98">
+        <v>0.73056994818652798</v>
+      </c>
+      <c r="D98">
+        <v>0.76165803108808205</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4">
+      <c r="A99" t="s">
+        <v>9</v>
+      </c>
+      <c r="B99">
+        <v>0.76683937823834103</v>
+      </c>
+      <c r="C99">
+        <v>0.75129533678756399</v>
+      </c>
+      <c r="D99">
+        <v>0.82383419689119097</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4">
+      <c r="A100" t="s">
+        <v>9</v>
+      </c>
+      <c r="B100">
+        <v>0.72020725388601003</v>
+      </c>
+      <c r="C100">
+        <v>0.78238341968911895</v>
+      </c>
+      <c r="D100">
+        <v>0.81347150259067302</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
+      <c r="A101" t="s">
+        <v>9</v>
+      </c>
+      <c r="B101">
+        <v>0.77720207253885998</v>
+      </c>
+      <c r="C101">
+        <v>0.78756476683937804</v>
+      </c>
+      <c r="D101">
+        <v>0.78238341968911895</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4">
+      <c r="A102" t="s">
+        <v>10</v>
+      </c>
+      <c r="B102">
+        <v>0.82157497303128302</v>
+      </c>
+      <c r="C102">
+        <v>0.809816612729234</v>
+      </c>
+      <c r="D102">
+        <v>0.85064724919093804</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4">
+      <c r="A103" t="s">
+        <v>10</v>
+      </c>
+      <c r="B103">
+        <v>0.83878101402373195</v>
+      </c>
+      <c r="C103">
+        <v>0.84363538295577101</v>
+      </c>
+      <c r="D103">
+        <v>0.85199568500539302</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4">
+      <c r="A104" t="s">
+        <v>10</v>
+      </c>
+      <c r="B104">
+        <v>0.85749730312837102</v>
+      </c>
+      <c r="C104">
+        <v>0.84848975188780995</v>
+      </c>
+      <c r="D104">
+        <v>0.857281553398058</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4">
+      <c r="A105" t="s">
+        <v>10</v>
+      </c>
+      <c r="B105">
+        <v>0.81569579288025895</v>
+      </c>
+      <c r="C105">
+        <v>0.84201725997842503</v>
+      </c>
+      <c r="D105">
+        <v>0.82804746494066805</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4">
+      <c r="A106" t="s">
+        <v>10</v>
+      </c>
+      <c r="B106">
+        <v>0.80717367853290101</v>
+      </c>
+      <c r="C106">
+        <v>0.82179072276159604</v>
+      </c>
+      <c r="D106">
+        <v>0.853883495145631</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4">
+      <c r="A107" t="s">
+        <v>10</v>
+      </c>
+      <c r="B107">
+        <v>0.85215749730312795</v>
+      </c>
+      <c r="C107">
+        <v>0.87443365695792796</v>
+      </c>
+      <c r="D107">
+        <v>0.87459546925566301</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4">
+      <c r="A108" t="s">
+        <v>10</v>
+      </c>
+      <c r="B108">
+        <v>0.79541531823085199</v>
+      </c>
+      <c r="C108">
+        <v>0.77087378640776605</v>
+      </c>
+      <c r="D108">
+        <v>0.877238403451995</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4">
+      <c r="A109" t="s">
+        <v>10</v>
+      </c>
+      <c r="B109">
+        <v>0.81790722761596502</v>
+      </c>
+      <c r="C109">
+        <v>0.80717367853290101</v>
+      </c>
+      <c r="D109">
+        <v>0.78867313915857595</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4">
+      <c r="A110" t="s">
+        <v>10</v>
+      </c>
+      <c r="B110">
+        <v>0.838403451995685</v>
+      </c>
+      <c r="C110">
+        <v>0.84358144552319303</v>
+      </c>
+      <c r="D110">
+        <v>0.81790722761596502</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4">
+      <c r="A111" t="s">
+        <v>10</v>
+      </c>
+      <c r="B111">
+        <v>0.87195253505933101</v>
+      </c>
+      <c r="C111">
+        <v>0.87400215749730303</v>
+      </c>
+      <c r="D111">
+        <v>0.83193096008629897</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4">
+      <c r="A112" t="s">
+        <v>10</v>
+      </c>
+      <c r="B112">
+        <v>0.82971952535059301</v>
+      </c>
+      <c r="C112">
+        <v>0.79546925566342996</v>
+      </c>
+      <c r="D112">
+        <v>0.842610571736785</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4">
+      <c r="A113" t="s">
+        <v>10</v>
+      </c>
+      <c r="B113">
+        <v>0.80102481121898494</v>
+      </c>
+      <c r="C113">
+        <v>0.83824163969794996</v>
+      </c>
+      <c r="D113">
+        <v>0.86127292340884498</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4">
+      <c r="A114" t="s">
+        <v>10</v>
+      </c>
+      <c r="B114">
+        <v>0.836569579288025</v>
+      </c>
+      <c r="C114">
+        <v>0.85091693635382903</v>
+      </c>
+      <c r="D114">
+        <v>0.81839266450916903</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4">
+      <c r="A115" t="s">
+        <v>10</v>
+      </c>
+      <c r="B115">
+        <v>0.86170442286947102</v>
+      </c>
+      <c r="C115">
+        <v>0.84649406688241602</v>
+      </c>
+      <c r="D115">
+        <v>0.85307443365695701</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4">
+      <c r="A116" t="s">
+        <v>10</v>
+      </c>
+      <c r="B116">
+        <v>0.82367853290183302</v>
+      </c>
+      <c r="C116">
+        <v>0.78629989212513396</v>
+      </c>
+      <c r="D116">
+        <v>0.87998921251348405</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
+      <c r="A117" t="s">
+        <v>10</v>
+      </c>
+      <c r="B117">
+        <v>0.82599784250269603</v>
+      </c>
+      <c r="C117">
+        <v>0.86477885652642905</v>
+      </c>
+      <c r="D117">
+        <v>0.84541531823085203</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4">
+      <c r="A118" t="s">
+        <v>10</v>
+      </c>
+      <c r="B118">
+        <v>0.78371089536138006</v>
+      </c>
+      <c r="C118">
+        <v>0.83991370010787403</v>
+      </c>
+      <c r="D118">
+        <v>0.85943905070118598</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4">
+      <c r="A119" t="s">
+        <v>10</v>
+      </c>
+      <c r="B119">
+        <v>0.81089536138079799</v>
+      </c>
+      <c r="C119">
+        <v>0.82599784250269603</v>
+      </c>
+      <c r="D119">
+        <v>0.87011866235167201</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4">
+      <c r="A120" t="s">
+        <v>10</v>
+      </c>
+      <c r="B120">
+        <v>0.86526429341963296</v>
+      </c>
+      <c r="C120">
+        <v>0.86612729234088404</v>
+      </c>
+      <c r="D120">
+        <v>0.85248112189859704</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4">
+      <c r="A121" t="s">
+        <v>10</v>
+      </c>
+      <c r="B121">
+        <v>0.84002157497303098</v>
+      </c>
+      <c r="C121">
+        <v>0.859654800431499</v>
+      </c>
+      <c r="D121">
+        <v>0.85641855447680604</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4">
+      <c r="A122" t="s">
+        <v>10</v>
+      </c>
+      <c r="B122">
+        <v>0.86272923408845703</v>
+      </c>
+      <c r="C122">
+        <v>0.89390507011866205</v>
+      </c>
+      <c r="D122">
+        <v>0.86461704422869401</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4">
+      <c r="A123" t="s">
+        <v>10</v>
+      </c>
+      <c r="B123">
+        <v>0.84115426105717295</v>
+      </c>
+      <c r="C123">
+        <v>0.85922330097087296</v>
+      </c>
+      <c r="D123">
+        <v>0.87259978425026896</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4">
+      <c r="A124" t="s">
+        <v>10</v>
+      </c>
+      <c r="B124">
+        <v>0.83149946062567404</v>
+      </c>
+      <c r="C124">
+        <v>0.87842502696871605</v>
+      </c>
+      <c r="D124">
+        <v>0.84314994606256699</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4">
+      <c r="A125" t="s">
+        <v>10</v>
+      </c>
+      <c r="B125">
+        <v>0.83387270765911503</v>
+      </c>
+      <c r="C125">
+        <v>0.85064724919093804</v>
+      </c>
+      <c r="D125">
+        <v>0.83387270765911503</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4">
+      <c r="A126" t="s">
+        <v>10</v>
+      </c>
+      <c r="B126">
+        <v>0.82405609492988097</v>
+      </c>
+      <c r="C126">
+        <v>0.83527508090614799</v>
+      </c>
+      <c r="D126">
+        <v>0.85382955771305202</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4">
+      <c r="A127" t="s">
+        <v>10</v>
+      </c>
+      <c r="B127">
+        <v>0.81521035598705405</v>
+      </c>
+      <c r="C127">
+        <v>0.83959007551240505</v>
+      </c>
+      <c r="D127">
+        <v>0.89687162891046301</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4">
+      <c r="A128" t="s">
+        <v>10</v>
+      </c>
+      <c r="B128">
+        <v>0.79600862998921196</v>
+      </c>
+      <c r="C128">
+        <v>0.805609492988133</v>
+      </c>
+      <c r="D128">
+        <v>0.82891046386192002</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4">
+      <c r="A129" t="s">
+        <v>10</v>
+      </c>
+      <c r="B129">
+        <v>0.81299892125134798</v>
+      </c>
+      <c r="C129">
+        <v>0.86170442286947102</v>
+      </c>
+      <c r="D129">
+        <v>0.86925566343042004</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4">
+      <c r="A130" t="s">
+        <v>10</v>
+      </c>
+      <c r="B130">
+        <v>0.80933117583602998</v>
+      </c>
+      <c r="C130">
+        <v>0.82065803667745396</v>
+      </c>
+      <c r="D130">
+        <v>0.84395900755123998</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4">
+      <c r="A131" t="s">
+        <v>10</v>
+      </c>
+      <c r="B131">
+        <v>0.81731391585760504</v>
+      </c>
+      <c r="C131">
+        <v>0.82880258899676296</v>
+      </c>
+      <c r="D131">
+        <v>0.88834951456310596</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4">
+      <c r="A132" t="s">
+        <v>10</v>
+      </c>
+      <c r="B132">
+        <v>0.83775620280474605</v>
+      </c>
+      <c r="C132">
+        <v>0.86208198489751797</v>
+      </c>
+      <c r="D132">
+        <v>0.84379719525350605</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4">
+      <c r="A133" t="s">
+        <v>10</v>
+      </c>
+      <c r="B133">
+        <v>0.84800431499460605</v>
+      </c>
+      <c r="C133">
+        <v>0.85933117583603003</v>
+      </c>
+      <c r="D133">
+        <v>0.84018338727076503</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4">
+      <c r="A134" t="s">
+        <v>10</v>
+      </c>
+      <c r="B134">
+        <v>0.79180151024811196</v>
+      </c>
+      <c r="C134">
+        <v>0.80933117583602998</v>
+      </c>
+      <c r="D134">
+        <v>0.895846817691477</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4">
+      <c r="A135" t="s">
+        <v>10</v>
+      </c>
+      <c r="B135">
+        <v>0.81774541531822997</v>
+      </c>
+      <c r="C135">
+        <v>0.82206040992448703</v>
+      </c>
+      <c r="D135">
+        <v>0.83570658036677403</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4">
+      <c r="A136" t="s">
+        <v>10</v>
+      </c>
+      <c r="B136">
+        <v>0.81014023732470297</v>
+      </c>
+      <c r="C136">
+        <v>0.84498381877022599</v>
+      </c>
+      <c r="D136">
+        <v>0.87944983818770195</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4">
+      <c r="A137" t="s">
+        <v>10</v>
+      </c>
+      <c r="B137">
+        <v>0.81040992448759397</v>
+      </c>
+      <c r="C137">
+        <v>0.84212513484358098</v>
+      </c>
+      <c r="D137">
+        <v>0.91035598705501597</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4">
+      <c r="A138" t="s">
+        <v>10</v>
+      </c>
+      <c r="B138">
+        <v>0.81666666666666599</v>
+      </c>
+      <c r="C138">
+        <v>0.86094929881337601</v>
+      </c>
+      <c r="D138">
+        <v>0.87637540453074403</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4">
+      <c r="A139" t="s">
+        <v>10</v>
+      </c>
+      <c r="B139">
+        <v>0.80755124056094896</v>
+      </c>
+      <c r="C139">
+        <v>0.85517799352750801</v>
+      </c>
+      <c r="D139">
+        <v>0.83489751887810104</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4">
+      <c r="A140" t="s">
+        <v>10</v>
+      </c>
+      <c r="B140">
+        <v>0.84045307443365602</v>
+      </c>
+      <c r="C140">
+        <v>0.84115426105717295</v>
+      </c>
+      <c r="D140">
+        <v>0.80976267529665502</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4">
+      <c r="A141" t="s">
+        <v>10</v>
+      </c>
+      <c r="B141">
+        <v>0.82211434735706501</v>
+      </c>
+      <c r="C141">
+        <v>0.83613807982739996</v>
+      </c>
+      <c r="D141">
+        <v>0.85086299892125095</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4">
+      <c r="A142" t="s">
+        <v>10</v>
+      </c>
+      <c r="B142">
+        <v>0.77195253505933104</v>
+      </c>
+      <c r="C142">
+        <v>0.79989212513484298</v>
+      </c>
+      <c r="D142">
+        <v>0.84606256742178998</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4">
+      <c r="A143" t="s">
+        <v>10</v>
+      </c>
+      <c r="B143">
+        <v>0.83516720604099204</v>
+      </c>
+      <c r="C143">
+        <v>0.84843581445523097</v>
+      </c>
+      <c r="D143">
+        <v>0.86262135922330097</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4">
+      <c r="A144" t="s">
+        <v>10</v>
+      </c>
+      <c r="B144">
+        <v>0.86779935275080899</v>
+      </c>
+      <c r="C144">
+        <v>0.86585760517799304</v>
+      </c>
+      <c r="D144">
+        <v>0.86488673139158501</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4">
+      <c r="A145" t="s">
+        <v>10</v>
+      </c>
+      <c r="B145">
+        <v>0.804045307443365</v>
+      </c>
+      <c r="C145">
+        <v>0.81850053937432499</v>
+      </c>
+      <c r="D145">
+        <v>0.85302049622437903</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4">
+      <c r="A146" t="s">
+        <v>10</v>
+      </c>
+      <c r="B146">
+        <v>0.86256742179072199</v>
+      </c>
+      <c r="C146">
+        <v>0.87184466019417395</v>
+      </c>
+      <c r="D146">
+        <v>0.86828478964401201</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4">
+      <c r="A147" t="s">
+        <v>10</v>
+      </c>
+      <c r="B147">
+        <v>0.87454153182308503</v>
+      </c>
+      <c r="C147">
+        <v>0.87594390507011799</v>
+      </c>
+      <c r="D147">
+        <v>0.81823085221143399</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4">
+      <c r="A148" t="s">
+        <v>10</v>
+      </c>
+      <c r="B148">
+        <v>0.87508090614886702</v>
+      </c>
+      <c r="C148">
+        <v>0.84940668824163901</v>
+      </c>
+      <c r="D148">
+        <v>0.84374325782092696</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4">
+      <c r="A149" t="s">
+        <v>10</v>
+      </c>
+      <c r="B149">
+        <v>0.85188781014023696</v>
+      </c>
+      <c r="C149">
+        <v>0.85005393743257796</v>
+      </c>
+      <c r="D149">
+        <v>0.865426105717367</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4">
+      <c r="A150" t="s">
+        <v>10</v>
+      </c>
+      <c r="B150">
+        <v>0.80507011866235101</v>
+      </c>
+      <c r="C150">
+        <v>0.82049622437971903</v>
+      </c>
+      <c r="D150">
+        <v>0.84536138079827405</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4">
+      <c r="A151" t="s">
+        <v>10</v>
+      </c>
+      <c r="B151">
+        <v>0.83872707659115397</v>
+      </c>
+      <c r="C151">
+        <v>0.85507011866235105</v>
+      </c>
+      <c r="D151">
+        <v>0.817421790722761</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4">
+      <c r="A152" t="s">
+        <v>10</v>
+      </c>
+      <c r="B152">
+        <v>0.86456310679611603</v>
+      </c>
+      <c r="C152">
+        <v>0.88220064724919001</v>
+      </c>
+      <c r="D152">
+        <v>0.829234088457389</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4">
+      <c r="A153" t="s">
+        <v>10</v>
+      </c>
+      <c r="B153">
+        <v>0.81720604099244798</v>
+      </c>
+      <c r="C153">
+        <v>0.83710895361380799</v>
+      </c>
+      <c r="D153">
+        <v>0.85765911542610496</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4">
+      <c r="A154" t="s">
+        <v>10</v>
+      </c>
+      <c r="B154">
+        <v>0.83117583603020495</v>
+      </c>
+      <c r="C154">
+        <v>0.82491909385113205</v>
+      </c>
+      <c r="D154">
+        <v>0.82437971952535005</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4">
+      <c r="A155" t="s">
+        <v>10</v>
+      </c>
+      <c r="B155">
+        <v>0.78667745415318202</v>
+      </c>
+      <c r="C155">
+        <v>0.84724919093851103</v>
+      </c>
+      <c r="D155">
+        <v>0.87335490830636398</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4">
+      <c r="A156" t="s">
+        <v>10</v>
+      </c>
+      <c r="B156">
+        <v>0.84552319309600799</v>
+      </c>
+      <c r="C156">
+        <v>0.87831715210355998</v>
+      </c>
+      <c r="D156">
+        <v>0.87761596548004295</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4">
+      <c r="A157" t="s">
+        <v>10</v>
+      </c>
+      <c r="B157">
+        <v>0.84217907227615896</v>
+      </c>
+      <c r="C157">
+        <v>0.84902912621359194</v>
+      </c>
+      <c r="D157">
+        <v>0.85517799352750801</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4">
+      <c r="A158" t="s">
+        <v>10</v>
+      </c>
+      <c r="B158">
+        <v>0.80102481121898605</v>
+      </c>
+      <c r="C158">
+        <v>0.82416396979503703</v>
+      </c>
+      <c r="D158">
+        <v>0.89870550161812301</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4">
+      <c r="A159" t="s">
+        <v>10</v>
+      </c>
+      <c r="B159">
+        <v>0.79751887810140198</v>
+      </c>
+      <c r="C159">
+        <v>0.82524271844660202</v>
+      </c>
+      <c r="D159">
+        <v>0.84919093851132699</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4">
+      <c r="A160" t="s">
+        <v>10</v>
+      </c>
+      <c r="B160">
+        <v>0.77799352750809003</v>
+      </c>
+      <c r="C160">
+        <v>0.82189859762675299</v>
+      </c>
+      <c r="D160">
+        <v>0.882740021574973</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4">
+      <c r="A161" t="s">
+        <v>10</v>
+      </c>
+      <c r="B161">
+        <v>0.82470334412081903</v>
+      </c>
+      <c r="C161">
+        <v>0.84169363538295505</v>
+      </c>
+      <c r="D161">
+        <v>0.82826321467098096</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4">
+      <c r="A162" t="s">
+        <v>10</v>
+      </c>
+      <c r="B162">
+        <v>0.83430420711974096</v>
+      </c>
+      <c r="C162">
+        <v>0.84163969795037696</v>
+      </c>
+      <c r="D162">
+        <v>0.87508090614886702</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4">
+      <c r="A163" t="s">
+        <v>10</v>
+      </c>
+      <c r="B163">
+        <v>0.84174757281553403</v>
+      </c>
+      <c r="C163">
+        <v>0.85026968716289097</v>
+      </c>
+      <c r="D163">
+        <v>0.87216828478964303</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4">
+      <c r="A164" t="s">
+        <v>10</v>
+      </c>
+      <c r="B164">
+        <v>0.81337648327939505</v>
+      </c>
+      <c r="C164">
+        <v>0.82740021574972999</v>
+      </c>
+      <c r="D164">
+        <v>0.86127292340884498</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4">
+      <c r="A165" t="s">
+        <v>10</v>
+      </c>
+      <c r="B165">
+        <v>0.832901833872707</v>
+      </c>
+      <c r="C165">
+        <v>0.86202804746493999</v>
+      </c>
+      <c r="D165">
+        <v>0.832632146709816</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4">
+      <c r="A166" t="s">
+        <v>10</v>
+      </c>
+      <c r="B166">
+        <v>0.83570658036677403</v>
+      </c>
+      <c r="C166">
+        <v>0.82837108953613803</v>
+      </c>
+      <c r="D166">
+        <v>0.89935275080906096</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4">
+      <c r="A167" t="s">
+        <v>10</v>
+      </c>
+      <c r="B167">
+        <v>0.86208198489751797</v>
+      </c>
+      <c r="C167">
+        <v>0.87259978425026896</v>
+      </c>
+      <c r="D167">
+        <v>0.82885652642934105</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4">
+      <c r="A168" t="s">
+        <v>10</v>
+      </c>
+      <c r="B168">
+        <v>0.80701186623516696</v>
+      </c>
+      <c r="C168">
+        <v>0.83036677454153096</v>
+      </c>
+      <c r="D168">
+        <v>0.83495145631067902</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4">
+      <c r="A169" t="s">
+        <v>10</v>
+      </c>
+      <c r="B169">
+        <v>0.84498381877022599</v>
+      </c>
+      <c r="C169">
+        <v>0.86143473570658002</v>
+      </c>
+      <c r="D169">
+        <v>0.86116504854368903</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4">
+      <c r="A170" t="s">
+        <v>10</v>
+      </c>
+      <c r="B170">
+        <v>0.786192017259978</v>
+      </c>
+      <c r="C170">
+        <v>0.80469255663430395</v>
+      </c>
+      <c r="D170">
+        <v>0.85911542610571701</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4">
+      <c r="A171" t="s">
+        <v>10</v>
+      </c>
+      <c r="B171">
+        <v>0.88306364617044197</v>
+      </c>
+      <c r="C171">
+        <v>0.87810140237324696</v>
+      </c>
+      <c r="D171">
+        <v>0.89093851132685997</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4">
+      <c r="A172" t="s">
+        <v>10</v>
+      </c>
+      <c r="B172">
+        <v>0.83667745415318195</v>
+      </c>
+      <c r="C172">
+        <v>0.85253505933117502</v>
+      </c>
+      <c r="D172">
+        <v>0.85631067961164997</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4">
+      <c r="A173" t="s">
+        <v>10</v>
+      </c>
+      <c r="B173">
+        <v>0.83484358144552295</v>
+      </c>
+      <c r="C173">
+        <v>0.85059331175835995</v>
+      </c>
+      <c r="D173">
+        <v>0.86531823085221105</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4">
+      <c r="A174" t="s">
+        <v>10</v>
+      </c>
+      <c r="B174">
+        <v>0.81251348435814397</v>
+      </c>
+      <c r="C174">
+        <v>0.76208198489751799</v>
+      </c>
+      <c r="D174">
+        <v>0.88376483279395901</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4">
+      <c r="A175" t="s">
+        <v>10</v>
+      </c>
+      <c r="B175">
+        <v>0.84746494066882405</v>
+      </c>
+      <c r="C175">
+        <v>0.836839266450917</v>
+      </c>
+      <c r="D175">
+        <v>0.85636461704422795</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4">
+      <c r="A176" t="s">
+        <v>10</v>
+      </c>
+      <c r="B176">
+        <v>0.83775620280474605</v>
+      </c>
+      <c r="C176">
+        <v>0.87810140237324696</v>
+      </c>
+      <c r="D176">
+        <v>0.83441208198489702</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4">
+      <c r="A177" t="s">
+        <v>10</v>
+      </c>
+      <c r="B177">
+        <v>0.82804746494066805</v>
+      </c>
+      <c r="C177">
+        <v>0.82966558791801504</v>
+      </c>
+      <c r="D177">
+        <v>0.89552319309600803</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4">
+      <c r="A178" t="s">
+        <v>10</v>
+      </c>
+      <c r="B178">
+        <v>0.83926645091693597</v>
+      </c>
+      <c r="C178">
+        <v>0.87518878101402298</v>
+      </c>
+      <c r="D178">
+        <v>0.84395900755123998</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4">
+      <c r="A179" t="s">
+        <v>10</v>
+      </c>
+      <c r="B179">
+        <v>0.81677454153182205</v>
+      </c>
+      <c r="C179">
+        <v>0.85361380798274</v>
+      </c>
+      <c r="D179">
+        <v>0.809546925566342</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4">
+      <c r="A180" t="s">
+        <v>10</v>
+      </c>
+      <c r="B180">
+        <v>0.80873786407767001</v>
+      </c>
+      <c r="C180">
+        <v>0.84169363538295505</v>
+      </c>
+      <c r="D180">
+        <v>0.90685005393743201</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4">
+      <c r="A181" t="s">
+        <v>10</v>
+      </c>
+      <c r="B181">
+        <v>0.84368932038834898</v>
+      </c>
+      <c r="C181">
+        <v>0.88327939590075499</v>
+      </c>
+      <c r="D181">
+        <v>0.86132686084142396</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4">
+      <c r="A182" t="s">
+        <v>10</v>
+      </c>
+      <c r="B182">
+        <v>0.83322545846817697</v>
+      </c>
+      <c r="C182">
+        <v>0.84913700107874801</v>
+      </c>
+      <c r="D182">
+        <v>0.87103559870550096</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4">
+      <c r="A183" t="s">
+        <v>10</v>
+      </c>
+      <c r="B183">
+        <v>0.79228694714131598</v>
+      </c>
+      <c r="C183">
+        <v>0.823462783171521</v>
+      </c>
+      <c r="D183">
+        <v>0.83279395900755104</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4">
+      <c r="A184" t="s">
+        <v>10</v>
+      </c>
+      <c r="B184">
+        <v>0.86785329018338697</v>
+      </c>
+      <c r="C184">
+        <v>0.86456310679611603</v>
+      </c>
+      <c r="D184">
+        <v>0.86235167206040897</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4">
+      <c r="A185" t="s">
+        <v>10</v>
+      </c>
+      <c r="B185">
+        <v>0.79320388349514503</v>
+      </c>
+      <c r="C185">
+        <v>0.80755124056094896</v>
+      </c>
+      <c r="D185">
+        <v>0.89676375404530695</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4">
+      <c r="A186" t="s">
+        <v>10</v>
+      </c>
+      <c r="B186">
+        <v>0.86051779935274997</v>
+      </c>
+      <c r="C186">
+        <v>0.85275080906148804</v>
+      </c>
+      <c r="D186">
+        <v>0.84644012944983804</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4">
+      <c r="A187" t="s">
+        <v>10</v>
+      </c>
+      <c r="B187">
+        <v>0.86445523193095997</v>
+      </c>
+      <c r="C187">
+        <v>0.880906148867314</v>
+      </c>
+      <c r="D187">
+        <v>0.87384034519956799</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4">
+      <c r="A188" t="s">
+        <v>10</v>
+      </c>
+      <c r="B188">
+        <v>0.82319309600863</v>
+      </c>
+      <c r="C188">
+        <v>0.84045307443365702</v>
+      </c>
+      <c r="D188">
+        <v>0.84018338727076503</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4">
+      <c r="A189" t="s">
+        <v>10</v>
+      </c>
+      <c r="B189">
+        <v>0.79439050701186598</v>
+      </c>
+      <c r="C189">
+        <v>0.80987055016181198</v>
+      </c>
+      <c r="D189">
+        <v>0.84131607335490799</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4">
+      <c r="A190" t="s">
+        <v>10</v>
+      </c>
+      <c r="B190">
+        <v>0.81467098166127205</v>
+      </c>
+      <c r="C190">
+        <v>0.82335490830636404</v>
+      </c>
+      <c r="D190">
+        <v>0.83451995685005398</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4">
+      <c r="A191" t="s">
+        <v>10</v>
+      </c>
+      <c r="B191">
+        <v>0.83419633225458401</v>
+      </c>
+      <c r="C191">
+        <v>0.83419633225458401</v>
+      </c>
+      <c r="D191">
+        <v>0.85587918015102404</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4">
+      <c r="A192" t="s">
+        <v>10</v>
+      </c>
+      <c r="B192">
+        <v>0.84228694714131602</v>
+      </c>
+      <c r="C192">
+        <v>0.83737864077669899</v>
+      </c>
+      <c r="D192">
+        <v>0.84881337648327904</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4">
+      <c r="A193" t="s">
+        <v>10</v>
+      </c>
+      <c r="B193">
+        <v>0.78861920172599798</v>
+      </c>
+      <c r="C193">
+        <v>0.82567421790722695</v>
+      </c>
+      <c r="D193">
+        <v>0.84714131607335497</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4">
+      <c r="A194" t="s">
+        <v>10</v>
+      </c>
+      <c r="B194">
+        <v>0.818985976267529</v>
+      </c>
+      <c r="C194">
+        <v>0.84919093851132599</v>
+      </c>
+      <c r="D194">
+        <v>0.84956850053937405</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4">
+      <c r="A195" t="s">
+        <v>10</v>
+      </c>
+      <c r="B195">
+        <v>0.87103559870550096</v>
+      </c>
+      <c r="C195">
+        <v>0.89778856526429296</v>
+      </c>
+      <c r="D195">
+        <v>0.81240560949298801</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4">
+      <c r="A196" t="s">
+        <v>10</v>
+      </c>
+      <c r="B196">
+        <v>0.85323624595469205</v>
+      </c>
+      <c r="C196">
+        <v>0.85895361380798196</v>
+      </c>
+      <c r="D196">
+        <v>0.85722761596548003</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4">
+      <c r="A197" t="s">
+        <v>10</v>
+      </c>
+      <c r="B197">
+        <v>0.78716289104638604</v>
+      </c>
+      <c r="C197">
+        <v>0.82696871628910396</v>
+      </c>
+      <c r="D197">
+        <v>0.85895361380798196</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4">
+      <c r="A198" t="s">
+        <v>10</v>
+      </c>
+      <c r="B198">
+        <v>0.85604099244875898</v>
+      </c>
+      <c r="C198">
+        <v>0.83020496224379703</v>
+      </c>
+      <c r="D198">
+        <v>0.83770226537216796</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4">
+      <c r="A199" t="s">
+        <v>10</v>
+      </c>
+      <c r="B199">
+        <v>0.81823085221143399</v>
+      </c>
+      <c r="C199">
+        <v>0.83381877022653705</v>
+      </c>
+      <c r="D199">
+        <v>0.87028047464940606</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4">
+      <c r="A200" t="s">
+        <v>10</v>
+      </c>
+      <c r="B200">
+        <v>0.80711974110032303</v>
+      </c>
+      <c r="C200">
+        <v>0.83635382955771298</v>
+      </c>
+      <c r="D200">
+        <v>0.87006472491909304</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4">
+      <c r="A201" t="s">
+        <v>10</v>
+      </c>
+      <c r="B201">
+        <v>0.81877022653721598</v>
+      </c>
+      <c r="C201">
+        <v>0.84476806903991297</v>
+      </c>
+      <c r="D201">
+        <v>0.86871628910463805</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4">
+      <c r="A202" t="s">
+        <v>11</v>
+      </c>
+      <c r="B202">
+        <v>0.855099401992238</v>
+      </c>
+      <c r="C202">
+        <v>0.84259669459526798</v>
+      </c>
+      <c r="D202">
+        <v>0.87504943986415595</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4">
+      <c r="A203" t="s">
+        <v>11</v>
+      </c>
+      <c r="B203">
+        <v>0.86434574983783297</v>
+      </c>
+      <c r="C203">
+        <v>0.88849890992871705</v>
+      </c>
+      <c r="D203">
+        <v>0.84197880419305504</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4">
+      <c r="A204" t="s">
+        <v>11</v>
+      </c>
+      <c r="B204">
+        <v>0.87517344633138505</v>
+      </c>
+      <c r="C204">
+        <v>0.86391538125349299</v>
+      </c>
+      <c r="D204">
+        <v>0.88000227165141398</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4">
+      <c r="A205" t="s">
+        <v>11</v>
+      </c>
+      <c r="B205">
+        <v>0.85003333967614503</v>
+      </c>
+      <c r="C205">
+        <v>0.86635941865675403</v>
+      </c>
+      <c r="D205">
+        <v>0.84647274479762702</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4">
+      <c r="A206" t="s">
+        <v>11</v>
+      </c>
+      <c r="B206">
+        <v>0.86112793339997196</v>
+      </c>
+      <c r="C206">
+        <v>0.87875247319285799</v>
+      </c>
+      <c r="D206">
+        <v>0.88033121078432996</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4">
+      <c r="A207" t="s">
+        <v>11</v>
+      </c>
+      <c r="B207">
+        <v>0.876013299572862</v>
+      </c>
+      <c r="C207">
+        <v>0.88723664242203903</v>
+      </c>
+      <c r="D207">
+        <v>0.89347571844987705</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4">
+      <c r="A208" t="s">
+        <v>11</v>
+      </c>
+      <c r="B208">
+        <v>0.84354915281595</v>
+      </c>
+      <c r="C208">
+        <v>0.80596288934403304</v>
+      </c>
+      <c r="D208">
+        <v>0.893713792481304</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4">
+      <c r="A209" t="s">
+        <v>11</v>
+      </c>
+      <c r="B209">
+        <v>0.83905114422722904</v>
+      </c>
+      <c r="C209">
+        <v>0.85939907920646297</v>
+      </c>
+      <c r="D209">
+        <v>0.81593694249604798</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4">
+      <c r="A210" t="s">
+        <v>11</v>
+      </c>
+      <c r="B210">
+        <v>0.86762360011461603</v>
+      </c>
+      <c r="C210">
+        <v>0.88142330536360203</v>
+      </c>
+      <c r="D210">
+        <v>0.83698026310681595</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4">
+      <c r="A211" t="s">
+        <v>11</v>
+      </c>
+      <c r="B211">
+        <v>0.90734998297503799</v>
+      </c>
+      <c r="C211">
+        <v>0.90203915843167704</v>
+      </c>
+      <c r="D211">
+        <v>0.86157877502763303</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4">
+      <c r="A212" t="s">
+        <v>11</v>
+      </c>
+      <c r="B212">
+        <v>0.84269448912275102</v>
+      </c>
+      <c r="C212">
+        <v>0.81188552894773303</v>
+      </c>
+      <c r="D212">
+        <v>0.85317232014337097</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4">
+      <c r="A213" t="s">
+        <v>11</v>
+      </c>
+      <c r="B213">
+        <v>0.82817788727867803</v>
+      </c>
+      <c r="C213">
+        <v>0.86985090148542699</v>
+      </c>
+      <c r="D213">
+        <v>0.89770401058390004</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4">
+      <c r="A214" t="s">
+        <v>11</v>
+      </c>
+      <c r="B214">
+        <v>0.85444722867775502</v>
+      </c>
+      <c r="C214">
+        <v>0.878715593847881</v>
+      </c>
+      <c r="D214">
+        <v>0.83329240951513095</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4">
+      <c r="A215" t="s">
+        <v>11</v>
+      </c>
+      <c r="B215">
+        <v>0.89352555170717696</v>
+      </c>
+      <c r="C215">
+        <v>0.86559683719969605</v>
+      </c>
+      <c r="D215">
+        <v>0.88477199592306199</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4">
+      <c r="A216" t="s">
+        <v>11</v>
+      </c>
+      <c r="B216">
+        <v>0.84540299538407004</v>
+      </c>
+      <c r="C216">
+        <v>0.82299129327984899</v>
+      </c>
+      <c r="D216">
+        <v>0.89296281286889401</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4">
+      <c r="A217" t="s">
+        <v>11</v>
+      </c>
+      <c r="B217">
+        <v>0.85876704912397905</v>
+      </c>
+      <c r="C217">
+        <v>0.89506143440691299</v>
+      </c>
+      <c r="D217">
+        <v>0.86689940552216105</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4">
+      <c r="A218" t="s">
+        <v>11</v>
+      </c>
+      <c r="B218">
+        <v>0.83795608252931797</v>
+      </c>
+      <c r="C218">
+        <v>0.88956386143845401</v>
+      </c>
+      <c r="D218">
+        <v>0.882480688689252</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4">
+      <c r="A219" t="s">
+        <v>11</v>
+      </c>
+      <c r="B219">
+        <v>0.85540514251220801</v>
+      </c>
+      <c r="C219">
+        <v>0.87411500000907405</v>
+      </c>
+      <c r="D219">
+        <v>0.877623210038596</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4">
+      <c r="A220" t="s">
+        <v>11</v>
+      </c>
+      <c r="B220">
+        <v>0.88612510087850904</v>
+      </c>
+      <c r="C220">
+        <v>0.88686855726110703</v>
+      </c>
+      <c r="D220">
+        <v>0.87283984717468299</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4">
+      <c r="A221" t="s">
+        <v>11</v>
+      </c>
+      <c r="B221">
+        <v>0.88665665458133502</v>
+      </c>
+      <c r="C221">
+        <v>0.89286575392032197</v>
+      </c>
+      <c r="D221">
+        <v>0.88342226847841199</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4">
+      <c r="A222" t="s">
+        <v>11</v>
+      </c>
+      <c r="B222">
+        <v>0.89051532321560201</v>
+      </c>
+      <c r="C222">
+        <v>0.91908701905435897</v>
+      </c>
+      <c r="D222">
+        <v>0.87767806762376299</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4">
+      <c r="A223" t="s">
+        <v>11</v>
+      </c>
+      <c r="B223">
+        <v>0.86319458726124398</v>
+      </c>
+      <c r="C223">
+        <v>0.88841690264581596</v>
+      </c>
+      <c r="D223">
+        <v>0.89452878272546898</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4">
+      <c r="A224" t="s">
+        <v>11</v>
+      </c>
+      <c r="B224">
+        <v>0.85739798805846401</v>
+      </c>
+      <c r="C224">
+        <v>0.91233931516655697</v>
+      </c>
+      <c r="D224">
+        <v>0.85851135893206798</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4">
+      <c r="A225" t="s">
+        <v>11</v>
+      </c>
+      <c r="B225">
+        <v>0.85096683217531099</v>
+      </c>
+      <c r="C225">
+        <v>0.86710344709583498</v>
+      </c>
+      <c r="D225">
+        <v>0.87378327258481903</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4">
+      <c r="A226" t="s">
+        <v>11</v>
+      </c>
+      <c r="B226">
+        <v>0.85279425670370901</v>
+      </c>
+      <c r="C226">
+        <v>0.86435311750633104</v>
+      </c>
+      <c r="D226">
+        <v>0.89493840884013298</v>
+      </c>
+    </row>
+    <row r="227" spans="1:4">
+      <c r="A227" t="s">
+        <v>11</v>
+      </c>
+      <c r="B227">
+        <v>0.84441370648437997</v>
+      </c>
+      <c r="C227">
+        <v>0.87986373287465203</v>
+      </c>
+      <c r="D227">
+        <v>0.92083007963454599</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4">
+      <c r="A228" t="s">
+        <v>11</v>
+      </c>
+      <c r="B228">
+        <v>0.83445193448583699</v>
+      </c>
+      <c r="C228">
+        <v>0.83615344792005697</v>
+      </c>
+      <c r="D228">
+        <v>0.83239007043955304</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4">
+      <c r="A229" t="s">
+        <v>11</v>
+      </c>
+      <c r="B229">
+        <v>0.83976706748475305</v>
+      </c>
+      <c r="C229">
+        <v>0.89080934301432901</v>
+      </c>
+      <c r="D229">
+        <v>0.89148956237551702</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4">
+      <c r="A230" t="s">
+        <v>11</v>
+      </c>
+      <c r="B230">
+        <v>0.85692555786160496</v>
+      </c>
+      <c r="C230">
+        <v>0.86997414756253999</v>
+      </c>
+      <c r="D230">
+        <v>0.85764709454274202</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4">
+      <c r="A231" t="s">
+        <v>11</v>
+      </c>
+      <c r="B231">
+        <v>0.85254980931603097</v>
+      </c>
+      <c r="C231">
+        <v>0.85169479338691101</v>
+      </c>
+      <c r="D231">
+        <v>0.90883835095968901</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4">
+      <c r="A232" t="s">
+        <v>11</v>
+      </c>
+      <c r="B232">
+        <v>0.87270010697661904</v>
+      </c>
+      <c r="C232">
+        <v>0.89219522238614402</v>
+      </c>
+      <c r="D232">
+        <v>0.878595432470476</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4">
+      <c r="A233" t="s">
+        <v>11</v>
+      </c>
+      <c r="B233">
+        <v>0.86277438252496896</v>
+      </c>
+      <c r="C233">
+        <v>0.88414004937794</v>
+      </c>
+      <c r="D233">
+        <v>0.85769465112100296</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4">
+      <c r="A234" t="s">
+        <v>11</v>
+      </c>
+      <c r="B234">
+        <v>0.81577198980978705</v>
+      </c>
+      <c r="C234">
+        <v>0.82674178189151304</v>
+      </c>
+      <c r="D234">
+        <v>0.88717776105510204</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4">
+      <c r="A235" t="s">
+        <v>11</v>
+      </c>
+      <c r="B235">
+        <v>0.86436265069706797</v>
+      </c>
+      <c r="C235">
+        <v>0.860388421047806</v>
+      </c>
+      <c r="D235">
+        <v>0.86796263050693501</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4">
+      <c r="A236" t="s">
+        <v>11</v>
+      </c>
+      <c r="B236">
+        <v>0.81903601797185399</v>
+      </c>
+      <c r="C236">
+        <v>0.85699192218323605</v>
+      </c>
+      <c r="D236">
+        <v>0.89861283968990202</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4">
+      <c r="A237" t="s">
+        <v>11</v>
+      </c>
+      <c r="B237">
+        <v>0.84570228846798001</v>
+      </c>
+      <c r="C237">
+        <v>0.87848239612197798</v>
+      </c>
+      <c r="D237">
+        <v>0.92710741536309504</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4">
+      <c r="A238" t="s">
+        <v>11</v>
+      </c>
+      <c r="B238">
+        <v>0.84820958511435096</v>
+      </c>
+      <c r="C238">
+        <v>0.86956274181429305</v>
+      </c>
+      <c r="D238">
+        <v>0.88662382176044097</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4">
+      <c r="A239" t="s">
+        <v>11</v>
+      </c>
+      <c r="B239">
+        <v>0.82636511296919801</v>
+      </c>
+      <c r="C239">
+        <v>0.864294992307307</v>
+      </c>
+      <c r="D239">
+        <v>0.83904596142620003</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4">
+      <c r="A240" t="s">
+        <v>11</v>
+      </c>
+      <c r="B240">
+        <v>0.86504011538578396</v>
+      </c>
+      <c r="C240">
+        <v>0.89224984252777095</v>
+      </c>
+      <c r="D240">
+        <v>0.81472000738838402</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4">
+      <c r="A241" t="s">
+        <v>11</v>
+      </c>
+      <c r="B241">
+        <v>0.85224275070850097</v>
+      </c>
+      <c r="C241">
+        <v>0.864450600655434</v>
+      </c>
+      <c r="D241">
+        <v>0.85922536071988598</v>
+      </c>
+    </row>
+    <row r="242" spans="1:4">
+      <c r="A242" t="s">
+        <v>11</v>
+      </c>
+      <c r="B242">
+        <v>0.789978163391998</v>
+      </c>
+      <c r="C242">
+        <v>0.83955223269364998</v>
+      </c>
+      <c r="D242">
+        <v>0.89298527407065098</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4">
+      <c r="A243" t="s">
+        <v>11</v>
+      </c>
+      <c r="B243">
+        <v>0.86651205978981805</v>
+      </c>
+      <c r="C243">
+        <v>0.85935841156787196</v>
+      </c>
+      <c r="D243">
+        <v>0.874079406294614</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4">
+      <c r="A244" t="s">
+        <v>11</v>
+      </c>
+      <c r="B244">
+        <v>0.88314635131570995</v>
+      </c>
+      <c r="C244">
+        <v>0.88279300149238904</v>
+      </c>
+      <c r="D244">
+        <v>0.89222327841889004</v>
+      </c>
+    </row>
+    <row r="245" spans="1:4">
+      <c r="A245" t="s">
+        <v>11</v>
+      </c>
+      <c r="B245">
+        <v>0.82688648879589699</v>
+      </c>
+      <c r="C245">
+        <v>0.84453531849596997</v>
+      </c>
+      <c r="D245">
+        <v>0.88471748801402805</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4">
+      <c r="A246" t="s">
+        <v>11</v>
+      </c>
+      <c r="B246">
+        <v>0.88891815335815705</v>
+      </c>
+      <c r="C246">
+        <v>0.89662457394407402</v>
+      </c>
+      <c r="D246">
+        <v>0.87171268247310896</v>
+      </c>
+    </row>
+    <row r="247" spans="1:4">
+      <c r="A247" t="s">
+        <v>11</v>
+      </c>
+      <c r="B247">
+        <v>0.90739167505227503</v>
+      </c>
+      <c r="C247">
+        <v>0.90542878599165799</v>
+      </c>
+      <c r="D247">
+        <v>0.82891713084151897</v>
+      </c>
+    </row>
+    <row r="248" spans="1:4">
+      <c r="A248" t="s">
+        <v>11</v>
+      </c>
+      <c r="B248">
+        <v>0.89610208639173194</v>
+      </c>
+      <c r="C248">
+        <v>0.86767596512383505</v>
+      </c>
+      <c r="D248">
+        <v>0.86185382275629496</v>
+      </c>
+    </row>
+    <row r="249" spans="1:4">
+      <c r="A249" t="s">
+        <v>11</v>
+      </c>
+      <c r="B249">
+        <v>0.87659081288414398</v>
+      </c>
+      <c r="C249">
+        <v>0.868389815687307</v>
+      </c>
+      <c r="D249">
+        <v>0.88766439697050803</v>
+      </c>
+    </row>
+    <row r="250" spans="1:4">
+      <c r="A250" t="s">
+        <v>11</v>
+      </c>
+      <c r="B250">
+        <v>0.83076435203713295</v>
+      </c>
+      <c r="C250">
+        <v>0.84822168051632696</v>
+      </c>
+      <c r="D250">
+        <v>0.85323307153232697</v>
+      </c>
+    </row>
+    <row r="251" spans="1:4">
+      <c r="A251" t="s">
+        <v>11</v>
+      </c>
+      <c r="B251">
+        <v>0.84860102376781499</v>
+      </c>
+      <c r="C251">
+        <v>0.88064726726249198</v>
+      </c>
+      <c r="D251">
+        <v>0.82852759783080698</v>
+      </c>
+    </row>
+    <row r="252" spans="1:4">
+      <c r="A252" t="s">
+        <v>11</v>
+      </c>
+      <c r="B252">
+        <v>0.89431762235116197</v>
+      </c>
+      <c r="C252">
+        <v>0.91196095361288798</v>
+      </c>
+      <c r="D252">
+        <v>0.84484175517581495</v>
+      </c>
+    </row>
+    <row r="253" spans="1:4">
+      <c r="A253" t="s">
+        <v>11</v>
+      </c>
+      <c r="B253">
+        <v>0.85204209475799897</v>
+      </c>
+      <c r="C253">
+        <v>0.85796320661625303</v>
+      </c>
+      <c r="D253">
+        <v>0.87367017207283404</v>
+      </c>
+    </row>
+    <row r="254" spans="1:4">
+      <c r="A254" t="s">
+        <v>11</v>
+      </c>
+      <c r="B254">
+        <v>0.85799082184974496</v>
+      </c>
+      <c r="C254">
+        <v>0.85255995265176798</v>
+      </c>
+      <c r="D254">
+        <v>0.83951092184607901</v>
+      </c>
+    </row>
+    <row r="255" spans="1:4">
+      <c r="A255" t="s">
+        <v>11</v>
+      </c>
+      <c r="B255">
+        <v>0.83004129483094402</v>
+      </c>
+      <c r="C255">
+        <v>0.86060033691678495</v>
+      </c>
+      <c r="D255">
+        <v>0.89551010979835399</v>
+      </c>
+    </row>
+    <row r="256" spans="1:4">
+      <c r="A256" t="s">
+        <v>11</v>
+      </c>
+      <c r="B256">
+        <v>0.87391747470647796</v>
+      </c>
+      <c r="C256">
+        <v>0.90120516096888903</v>
+      </c>
+      <c r="D256">
+        <v>0.88258517492357502</v>
+      </c>
+    </row>
+    <row r="257" spans="1:4">
+      <c r="A257" t="s">
+        <v>11</v>
+      </c>
+      <c r="B257">
+        <v>0.85245889943514697</v>
+      </c>
+      <c r="C257">
+        <v>0.86520491375002195</v>
+      </c>
+      <c r="D257">
+        <v>0.87506888658714099</v>
+      </c>
+    </row>
+    <row r="258" spans="1:4">
+      <c r="A258" t="s">
+        <v>11</v>
+      </c>
+      <c r="B258">
+        <v>0.84187857900830998</v>
+      </c>
+      <c r="C258">
+        <v>0.85677841159722801</v>
+      </c>
+      <c r="D258">
+        <v>0.908838623146628</v>
+      </c>
+    </row>
+    <row r="259" spans="1:4">
+      <c r="A259" t="s">
+        <v>11</v>
+      </c>
+      <c r="B259">
+        <v>0.85853382025504998</v>
+      </c>
+      <c r="C259">
+        <v>0.87266816786006396</v>
+      </c>
+      <c r="D259">
+        <v>0.86262143874514896</v>
+      </c>
+    </row>
+    <row r="260" spans="1:4">
+      <c r="A260" t="s">
+        <v>11</v>
+      </c>
+      <c r="B260">
+        <v>0.82588881549406401</v>
+      </c>
+      <c r="C260">
+        <v>0.85869522726477399</v>
+      </c>
+      <c r="D260">
+        <v>0.90903273393970996</v>
+      </c>
+    </row>
+    <row r="261" spans="1:4">
+      <c r="A261" t="s">
+        <v>11</v>
+      </c>
+      <c r="B261">
+        <v>0.86515426212449797</v>
+      </c>
+      <c r="C261">
+        <v>0.86915091034701997</v>
+      </c>
+      <c r="D261">
+        <v>0.85015262334699604</v>
+      </c>
+    </row>
+    <row r="262" spans="1:4">
+      <c r="A262" t="s">
+        <v>11</v>
+      </c>
+      <c r="B262">
+        <v>0.87077918987742498</v>
+      </c>
+      <c r="C262">
+        <v>0.88587526145777096</v>
+      </c>
+      <c r="D262">
+        <v>0.87939277515120995</v>
+      </c>
+    </row>
+    <row r="263" spans="1:4">
+      <c r="A263" t="s">
+        <v>11</v>
+      </c>
+      <c r="B263">
+        <v>0.85918050358717402</v>
+      </c>
+      <c r="C263">
+        <v>0.84699459725939596</v>
+      </c>
+      <c r="D263">
+        <v>0.88699415608298404</v>
+      </c>
+    </row>
+    <row r="264" spans="1:4">
+      <c r="A264" t="s">
+        <v>11</v>
+      </c>
+      <c r="B264">
+        <v>0.86120607235540703</v>
+      </c>
+      <c r="C264">
+        <v>0.85806129900920602</v>
+      </c>
+      <c r="D264">
+        <v>0.88082639112095495</v>
+      </c>
+    </row>
+    <row r="265" spans="1:4">
+      <c r="A265" t="s">
+        <v>11</v>
+      </c>
+      <c r="B265">
+        <v>0.84785087840249695</v>
+      </c>
+      <c r="C265">
+        <v>0.89043665996578003</v>
+      </c>
+      <c r="D265">
+        <v>0.85550447641059202</v>
+      </c>
+    </row>
+    <row r="266" spans="1:4">
+      <c r="A266" t="s">
+        <v>11</v>
+      </c>
+      <c r="B266">
+        <v>0.87405822502959096</v>
+      </c>
+      <c r="C266">
+        <v>0.87251787142085802</v>
+      </c>
+      <c r="D266">
+        <v>0.903952496433584</v>
+      </c>
+    </row>
+    <row r="267" spans="1:4">
+      <c r="A267" t="s">
+        <v>11</v>
+      </c>
+      <c r="B267">
+        <v>0.894773980451673</v>
+      </c>
+      <c r="C267">
+        <v>0.90184171539541402</v>
+      </c>
+      <c r="D267">
+        <v>0.85223612346478805</v>
+      </c>
+    </row>
+    <row r="268" spans="1:4">
+      <c r="A268" t="s">
+        <v>11</v>
+      </c>
+      <c r="B268">
+        <v>0.83925401224437202</v>
+      </c>
+      <c r="C268">
+        <v>0.86795022506630504</v>
+      </c>
+      <c r="D268">
+        <v>0.85467787214163504</v>
+      </c>
+    </row>
+    <row r="269" spans="1:4">
+      <c r="A269" t="s">
+        <v>11</v>
+      </c>
+      <c r="B269">
+        <v>0.87587397081019602</v>
+      </c>
+      <c r="C269">
+        <v>0.89278795212175399</v>
+      </c>
+      <c r="D269">
+        <v>0.88374368528685898</v>
+      </c>
+    </row>
+    <row r="270" spans="1:4">
+      <c r="A270" t="s">
+        <v>11</v>
+      </c>
+      <c r="B270">
+        <v>0.84333968890530198</v>
+      </c>
+      <c r="C270">
+        <v>0.84553974237651097</v>
+      </c>
+      <c r="D270">
+        <v>0.900160312370891</v>
+      </c>
+    </row>
+    <row r="271" spans="1:4">
+      <c r="A271" t="s">
+        <v>11</v>
+      </c>
+      <c r="B271">
+        <v>0.89183376348907595</v>
+      </c>
+      <c r="C271">
+        <v>0.88637224332465203</v>
+      </c>
+      <c r="D271">
+        <v>0.902604226669944</v>
+      </c>
+    </row>
+    <row r="272" spans="1:4">
+      <c r="A272" t="s">
+        <v>11</v>
+      </c>
+      <c r="B272">
+        <v>0.876296435398767</v>
+      </c>
+      <c r="C272">
+        <v>0.88741478412371999</v>
+      </c>
+      <c r="D272">
+        <v>0.88763974175479399</v>
+      </c>
+    </row>
+    <row r="273" spans="1:4">
+      <c r="A273" t="s">
+        <v>11</v>
+      </c>
+      <c r="B273">
+        <v>0.87010797598953105</v>
+      </c>
+      <c r="C273">
+        <v>0.87957817990402898</v>
+      </c>
+      <c r="D273">
+        <v>0.89251297430762699</v>
+      </c>
+    </row>
+    <row r="274" spans="1:4">
+      <c r="A274" t="s">
+        <v>11</v>
+      </c>
+      <c r="B274">
+        <v>0.82890426310540299</v>
+      </c>
+      <c r="C274">
+        <v>0.80689737953682905</v>
+      </c>
+      <c r="D274">
+        <v>0.91436097471674405</v>
+      </c>
+    </row>
+    <row r="275" spans="1:4">
+      <c r="A275" t="s">
+        <v>11</v>
+      </c>
+      <c r="B275">
+        <v>0.87483738575945602</v>
+      </c>
+      <c r="C275">
+        <v>0.86070624137549401</v>
+      </c>
+      <c r="D275">
+        <v>0.86849744816630403</v>
+      </c>
+    </row>
+    <row r="276" spans="1:4">
+      <c r="A276" t="s">
+        <v>11</v>
+      </c>
+      <c r="B276">
+        <v>0.87350572978921903</v>
+      </c>
+      <c r="C276">
+        <v>0.90441779443985204</v>
+      </c>
+      <c r="D276">
+        <v>0.81919502399067301</v>
+      </c>
+    </row>
+    <row r="277" spans="1:4">
+      <c r="A277" t="s">
+        <v>11</v>
+      </c>
+      <c r="B277">
+        <v>0.84432180464853801</v>
+      </c>
+      <c r="C277">
+        <v>0.87050509577676505</v>
+      </c>
+      <c r="D277">
+        <v>0.912255756515995</v>
+      </c>
+    </row>
+    <row r="278" spans="1:4">
+      <c r="A278" t="s">
+        <v>11</v>
+      </c>
+      <c r="B278">
+        <v>0.86363032910986404</v>
+      </c>
+      <c r="C278">
+        <v>0.88513739111291301</v>
+      </c>
+      <c r="D278">
+        <v>0.85529876000730198</v>
+      </c>
+    </row>
+    <row r="279" spans="1:4">
+      <c r="A279" t="s">
+        <v>11</v>
+      </c>
+      <c r="B279">
+        <v>0.84749209550327598</v>
+      </c>
+      <c r="C279">
+        <v>0.88809453582261499</v>
+      </c>
+      <c r="D279">
+        <v>0.83012912852831</v>
+      </c>
+    </row>
+    <row r="280" spans="1:4">
+      <c r="A280" t="s">
+        <v>11</v>
+      </c>
+      <c r="B280">
+        <v>0.84862973578686496</v>
+      </c>
+      <c r="C280">
+        <v>0.87719451454095998</v>
+      </c>
+      <c r="D280">
+        <v>0.92789994263151299</v>
+      </c>
+    </row>
+    <row r="281" spans="1:4">
+      <c r="A281" t="s">
+        <v>11</v>
+      </c>
+      <c r="B281">
+        <v>0.86714461448890101</v>
+      </c>
+      <c r="C281">
+        <v>0.90356886338514097</v>
+      </c>
+      <c r="D281">
+        <v>0.88984677746896501</v>
+      </c>
+    </row>
+    <row r="282" spans="1:4">
+      <c r="A282" t="s">
+        <v>11</v>
+      </c>
+      <c r="B282">
+        <v>0.86410505758822997</v>
+      </c>
+      <c r="C282">
+        <v>0.87940363995148396</v>
+      </c>
+      <c r="D282">
+        <v>0.89693873740545604</v>
+      </c>
+    </row>
+    <row r="283" spans="1:4">
+      <c r="A283" t="s">
+        <v>11</v>
+      </c>
+      <c r="B283">
+        <v>0.81606669919376196</v>
+      </c>
+      <c r="C283">
+        <v>0.85450765435547604</v>
+      </c>
+      <c r="D283">
+        <v>0.85283380965516598</v>
+      </c>
+    </row>
+    <row r="284" spans="1:4">
+      <c r="A284" t="s">
+        <v>11</v>
+      </c>
+      <c r="B284">
+        <v>0.88522005281921801</v>
+      </c>
+      <c r="C284">
+        <v>0.88968218806645605</v>
+      </c>
+      <c r="D284">
+        <v>0.88497257195488399</v>
+      </c>
+    </row>
+    <row r="285" spans="1:4">
+      <c r="A285" t="s">
+        <v>11</v>
+      </c>
+      <c r="B285">
+        <v>0.82645304024796196</v>
+      </c>
+      <c r="C285">
+        <v>0.85153305170048699</v>
+      </c>
+      <c r="D285">
+        <v>0.92305799817749201</v>
+      </c>
+    </row>
+    <row r="286" spans="1:4">
+      <c r="A286" t="s">
+        <v>11</v>
+      </c>
+      <c r="B286">
+        <v>0.86265361541958896</v>
+      </c>
+      <c r="C286">
+        <v>0.86765582741698699</v>
+      </c>
+      <c r="D286">
+        <v>0.87350113653376305</v>
+      </c>
+    </row>
+    <row r="287" spans="1:4">
+      <c r="A287" t="s">
+        <v>11</v>
+      </c>
+      <c r="B287">
+        <v>0.89543880447229995</v>
+      </c>
+      <c r="C287">
+        <v>0.90715178163566101</v>
+      </c>
+      <c r="D287">
+        <v>0.89376523531653496</v>
+      </c>
+    </row>
+    <row r="288" spans="1:4">
+      <c r="A288" t="s">
+        <v>11</v>
+      </c>
+      <c r="B288">
+        <v>0.86731454738716895</v>
+      </c>
+      <c r="C288">
+        <v>0.87964778610788597</v>
+      </c>
+      <c r="D288">
+        <v>0.84935173562336197</v>
+      </c>
+    </row>
+    <row r="289" spans="1:4">
+      <c r="A289" t="s">
+        <v>11</v>
+      </c>
+      <c r="B289">
+        <v>0.82875675656626702</v>
+      </c>
+      <c r="C289">
+        <v>0.83490482331081195</v>
+      </c>
+      <c r="D289">
+        <v>0.87536149488625603</v>
+      </c>
+    </row>
+    <row r="290" spans="1:4">
+      <c r="A290" t="s">
+        <v>11</v>
+      </c>
+      <c r="B290">
+        <v>0.85108087714785197</v>
+      </c>
+      <c r="C290">
+        <v>0.85902962719784204</v>
+      </c>
+      <c r="D290">
+        <v>0.85038457748378005</v>
+      </c>
+    </row>
+    <row r="291" spans="1:4">
+      <c r="A291" t="s">
+        <v>11</v>
+      </c>
+      <c r="B291">
+        <v>0.85003995933404497</v>
+      </c>
+      <c r="C291">
+        <v>0.86251264064086197</v>
+      </c>
+      <c r="D291">
+        <v>0.87202717595428103</v>
+      </c>
+    </row>
+    <row r="292" spans="1:4">
+      <c r="A292" t="s">
+        <v>11</v>
+      </c>
+      <c r="B292">
+        <v>0.87972288108989805</v>
+      </c>
+      <c r="C292">
+        <v>0.86984083749864005</v>
+      </c>
+      <c r="D292">
+        <v>0.85688682655737802</v>
+      </c>
+    </row>
+    <row r="293" spans="1:4">
+      <c r="A293" t="s">
+        <v>11</v>
+      </c>
+      <c r="B293">
+        <v>0.830029446605965</v>
+      </c>
+      <c r="C293">
+        <v>0.84667401825464506</v>
+      </c>
+      <c r="D293">
+        <v>0.84193201892065395</v>
+      </c>
+    </row>
+    <row r="294" spans="1:4">
+      <c r="A294" t="s">
+        <v>11</v>
+      </c>
+      <c r="B294">
+        <v>0.84149288936711097</v>
+      </c>
+      <c r="C294">
+        <v>0.86350992798137904</v>
+      </c>
+      <c r="D294">
+        <v>0.87291216052277598</v>
+      </c>
+    </row>
+    <row r="295" spans="1:4">
+      <c r="A295" t="s">
+        <v>11</v>
+      </c>
+      <c r="B295">
+        <v>0.89708861104076099</v>
+      </c>
+      <c r="C295">
+        <v>0.91751287496631795</v>
+      </c>
+      <c r="D295">
+        <v>0.83988222694871095</v>
+      </c>
+    </row>
+    <row r="296" spans="1:4">
+      <c r="A296" t="s">
+        <v>11</v>
+      </c>
+      <c r="B296">
+        <v>0.87512033397165701</v>
+      </c>
+      <c r="C296">
+        <v>0.84965594745046602</v>
+      </c>
+      <c r="D296">
+        <v>0.89347214776741102</v>
+      </c>
+    </row>
+    <row r="297" spans="1:4">
+      <c r="A297" t="s">
+        <v>11</v>
+      </c>
+      <c r="B297">
+        <v>0.81211939594280103</v>
+      </c>
+      <c r="C297">
+        <v>0.84913839465871899</v>
+      </c>
+      <c r="D297">
+        <v>0.86428111194130897</v>
+      </c>
+    </row>
+    <row r="298" spans="1:4">
+      <c r="A298" t="s">
+        <v>11</v>
+      </c>
+      <c r="B298">
+        <v>0.87395192222719698</v>
+      </c>
+      <c r="C298">
+        <v>0.865083149716671</v>
+      </c>
+      <c r="D298">
+        <v>0.86968962235238401</v>
+      </c>
+    </row>
+    <row r="299" spans="1:4">
+      <c r="A299" t="s">
+        <v>11</v>
+      </c>
+      <c r="B299">
+        <v>0.86203986073666306</v>
+      </c>
+      <c r="C299">
+        <v>0.87226069816014895</v>
+      </c>
+      <c r="D299">
+        <v>0.88909778912322901</v>
+      </c>
+    </row>
+    <row r="300" spans="1:4">
+      <c r="A300" t="s">
+        <v>11</v>
+      </c>
+      <c r="B300">
+        <v>0.84055044453524796</v>
+      </c>
+      <c r="C300">
+        <v>0.86060729843176498</v>
+      </c>
+      <c r="D300">
+        <v>0.90205540251452798</v>
+      </c>
+    </row>
+    <row r="301" spans="1:4">
+      <c r="A301" t="s">
+        <v>11</v>
+      </c>
+      <c r="B301">
+        <v>0.84880833246140697</v>
+      </c>
+      <c r="C301">
+        <v>0.87887093813597905</v>
+      </c>
+      <c r="D301">
+        <v>0.88155070608655395</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>